<commit_message>
Auto update RUP 2026-10-20 10:02:12
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-10-20).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-10-20).xlsx
@@ -523,10 +523,10 @@
         <v>3445475044</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>799661284</v>
+        <v>0</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>4</v>
@@ -535,16 +535,16 @@
         <v>946739000</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>77</v>
+        <v>4</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>1746400284</v>
+        <v>946739000</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>-1699074760</v>
+        <v>-2498736044</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>50.68677792460598</v>
+        <v>27.4777494513758</v>
       </c>
     </row>
     <row r="3">
@@ -560,10 +560,10 @@
         <v>1573461786</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>812087786</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0</v>
@@ -572,16 +572,16 @@
         <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>812087786</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>-761374000</v>
+        <v>-1573461786</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>51.61153535634706</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -597,10 +597,10 @@
         <v>1385846979</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1385846979</v>
+        <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0</v>
@@ -609,16 +609,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1385846979</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0</v>
+        <v>-1385846979</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -634,10 +634,10 @@
         <v>1363592000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1363592000</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
@@ -646,16 +646,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1363592000</v>
+        <v>0</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0</v>
+        <v>-1363592000</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -708,10 +708,10 @@
         <v>3525770642</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>2497840402</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>5</v>
@@ -720,16 +720,16 @@
         <v>1027930240</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>103</v>
+        <v>5</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>3525770642</v>
+        <v>1027930240</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0</v>
+        <v>-2497840402</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>100</v>
+        <v>29.15476769121047</v>
       </c>
     </row>
     <row r="8">
@@ -745,10 +745,10 @@
         <v>1145858598</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>127</v>
+        <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1145858598</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
@@ -757,16 +757,16 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>127</v>
+        <v>0</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>1145858598</v>
+        <v>0</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0</v>
+        <v>-1145858598</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -856,10 +856,10 @@
         <v>3803059695</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2664973989</v>
+        <v>0</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0</v>
@@ -868,16 +868,16 @@
         <v>0</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>2664973989</v>
+        <v>0</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>-1138085706</v>
+        <v>-3803059695</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>70.07447168141283</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -893,10 +893,10 @@
         <v>985193227</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>892817964</v>
+        <v>0</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0</v>
@@ -905,16 +905,16 @@
         <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>892817964</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>-92375263</v>
+        <v>-985193227</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>90.62364006690436</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -967,10 +967,10 @@
         <v>27966252800</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>4961498888</v>
+        <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>0</v>
@@ -979,16 +979,16 @@
         <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>4961498888</v>
+        <v>0</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>-23004753912</v>
+        <v>-27966252800</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>17.74102137845225</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1041,10 +1041,10 @@
         <v>4398271129</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>4293942679</v>
+        <v>0</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>0</v>
@@ -1053,16 +1053,16 @@
         <v>0</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>4293942679</v>
+        <v>0</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>-104328450</v>
+        <v>-4398271129</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>97.62796683196471</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1078,10 +1078,10 @@
         <v>19312615339</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>162</v>
+        <v>0</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>18065133242</v>
+        <v>0</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>162</v>
+        <v>0</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>18065133242</v>
+        <v>0</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>-1247482097</v>
+        <v>-19312615339</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>93.54058435327075</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1115,10 +1115,10 @@
         <v>2386017478</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>2326664178</v>
+        <v>0</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>0</v>
@@ -1127,16 +1127,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>2326664178</v>
+        <v>0</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>-59353300</v>
+        <v>-2386017478</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>97.51245325957332</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1152,10 +1152,10 @@
         <v>26765831792</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>440</v>
+        <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>112381136563</v>
+        <v>0</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>1</v>
@@ -1164,16 +1164,16 @@
         <v>35000000</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>441</v>
+        <v>1</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>112416136563</v>
+        <v>35000000</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>85650304771</v>
+        <v>-26730831792</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>419.9986663466962</v>
+        <v>0.1307637299374387</v>
       </c>
     </row>
     <row r="20">
@@ -1189,10 +1189,10 @@
         <v>1187854402</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2122940502</v>
+        <v>0</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>0</v>
@@ -1201,16 +1201,16 @@
         <v>0</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>2122940502</v>
+        <v>0</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>935086100</v>
+        <v>-1187854402</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>178.7205989577164</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1263,10 +1263,10 @@
         <v>4670181047</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>1712312836</v>
+        <v>0</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>0</v>
@@ -1275,16 +1275,16 @@
         <v>0</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>1712312836</v>
+        <v>0</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>-2957868211</v>
+        <v>-4670181047</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>36.66480632693981</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1300,10 +1300,10 @@
         <v>9426756999</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>2146723107</v>
+        <v>0</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0</v>
@@ -1312,16 +1312,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>2146723107</v>
+        <v>0</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>-7280033892</v>
+        <v>-9426756999</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>22.77265773614114</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1337,10 +1337,10 @@
         <v>762843197</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>613888229</v>
+        <v>0</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>0</v>
@@ -1349,16 +1349,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>613888229</v>
+        <v>0</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>-148954968</v>
+        <v>-762843197</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>80.47371090339553</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1374,10 +1374,10 @@
         <v>30934229421</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>297</v>
+        <v>0</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>9626894303</v>
+        <v>0</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>30</v>
@@ -1386,16 +1386,16 @@
         <v>52187493800</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>327</v>
+        <v>30</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>61814388103</v>
+        <v>52187493800</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>30880158682</v>
+        <v>21253264379</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>199.8252074158237</v>
+        <v>168.7046833776051</v>
       </c>
     </row>
     <row r="26">
@@ -1411,10 +1411,10 @@
         <v>10689556601</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>10689556601</v>
+        <v>0</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0</v>
@@ -1423,16 +1423,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>10689556601</v>
+        <v>0</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0</v>
+        <v>-10689556601</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1448,10 +1448,10 @@
         <v>3526787281</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>131</v>
+        <v>0</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>8063419229</v>
+        <v>0</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0</v>
@@ -1460,16 +1460,16 @@
         <v>0</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>131</v>
+        <v>0</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>8063419229</v>
+        <v>0</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>4536631948</v>
+        <v>-3526787281</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>228.6335575848415</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1485,10 +1485,10 @@
         <v>5579913725</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>122</v>
+        <v>0</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>11165380839</v>
+        <v>0</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0</v>
@@ -1497,16 +1497,16 @@
         <v>0</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>122</v>
+        <v>0</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>11165380839</v>
+        <v>0</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>5585467114</v>
+        <v>-5579913725</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>200.0995246391556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1522,10 +1522,10 @@
         <v>607018311</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>535177291</v>
+        <v>0</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>535177291</v>
+        <v>0</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>-71841020</v>
+        <v>-607018311</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>88.16493362751294</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1559,10 +1559,10 @@
         <v>6989299594</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>151</v>
+        <v>0</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>11325957961</v>
+        <v>0</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>2</v>
@@ -1571,16 +1571,16 @@
         <v>275000000</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>153</v>
+        <v>2</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>11600957961</v>
+        <v>275000000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>4611658367</v>
+        <v>-6714299594</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>165.9816953755839</v>
+        <v>3.934585952447583</v>
       </c>
     </row>
     <row r="31">
@@ -1596,10 +1596,10 @@
         <v>1781989871</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>312</v>
+        <v>0</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>32482515490</v>
+        <v>0</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0</v>
@@ -1608,16 +1608,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>312</v>
+        <v>0</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>32482515490</v>
+        <v>0</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>30700525619</v>
+        <v>-1781989871</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>1822.822678098152</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1670,10 +1670,10 @@
         <v>2401856856</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>1787561232</v>
+        <v>0</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0</v>
@@ -1682,16 +1682,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>1787561232</v>
+        <v>0</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>-614295624</v>
+        <v>-2401856856</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>74.42413678960726</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1707,10 +1707,10 @@
         <v>2150571134</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>1353030681</v>
+        <v>0</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>0</v>
@@ -1719,16 +1719,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>1353030681</v>
+        <v>0</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>-797540453</v>
+        <v>-2150571134</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>62.91494662087286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1744,10 +1744,10 @@
         <v>7783601090</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>1564313084</v>
+        <v>0</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0</v>
@@ -1756,16 +1756,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>1564313084</v>
+        <v>0</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>-6219288006</v>
+        <v>-7783601090</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>20.09754952639794</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1781,10 +1781,10 @@
         <v>5082238023</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>5082238023</v>
+        <v>0</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0</v>
@@ -1793,16 +1793,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>5082238023</v>
+        <v>0</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0</v>
+        <v>-5082238023</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1818,10 +1818,10 @@
         <v>3494926432</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>4568180877</v>
+        <v>0</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>3</v>
@@ -1830,16 +1830,16 @@
         <v>112860000</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>191</v>
+        <v>3</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>4681040877</v>
+        <v>112860000</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>1186114445</v>
+        <v>-3382066432</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>133.9381806191908</v>
+        <v>3.229252523504907</v>
       </c>
     </row>
     <row r="38">
@@ -1855,10 +1855,10 @@
         <v>465249566</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>465249566</v>
+        <v>0</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>0</v>
@@ -1867,16 +1867,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>465249566</v>
+        <v>0</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0</v>
+        <v>-465249566</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1892,10 +1892,10 @@
         <v>866968514</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>767266958</v>
+        <v>0</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0</v>
@@ -1904,16 +1904,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>767266958</v>
+        <v>0</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>-99701556</v>
+        <v>-866968514</v>
       </c>
       <c r="K39" s="4" t="n">
-        <v>88.49997959672154</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1929,10 +1929,10 @@
         <v>1439107189</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>758839698</v>
+        <v>0</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>5</v>
@@ -1941,16 +1941,16 @@
         <v>168247302</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>106</v>
+        <v>5</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>927087000</v>
+        <v>168247302</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>-512020189</v>
+        <v>-1270859887</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>64.42098316833577</v>
+        <v>11.6910889811419</v>
       </c>
     </row>
     <row r="41">
@@ -1966,10 +1966,10 @@
         <v>312595476</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>312595476</v>
+        <v>0</v>
       </c>
       <c r="F41" s="3" t="n">
         <v>0</v>
@@ -1978,16 +1978,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>312595476</v>
+        <v>0</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0</v>
+        <v>-312595476</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2003,10 +2003,10 @@
         <v>219851775</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>219851775</v>
+        <v>0</v>
       </c>
       <c r="F42" s="3" t="n">
         <v>0</v>
@@ -2015,16 +2015,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>219851775</v>
+        <v>0</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0</v>
+        <v>-219851775</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -2558,10 +2558,10 @@
         <v>2670750030</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>2639850030</v>
+        <v>0</v>
       </c>
       <c r="F57" s="3" t="n">
         <v>3</v>
@@ -2570,16 +2570,16 @@
         <v>30900000</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="I57" s="3" t="n">
-        <v>2670750030</v>
+        <v>30900000</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>0</v>
+        <v>-2639850030</v>
       </c>
       <c r="K57" s="4" t="n">
-        <v>100</v>
+        <v>1.156978363864326</v>
       </c>
     </row>
     <row r="58">
@@ -2743,10 +2743,10 @@
         <v>2845031415</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>1833404405</v>
+        <v>0</v>
       </c>
       <c r="F62" s="3" t="n">
         <v>1</v>
@@ -2755,16 +2755,16 @@
         <v>116900000</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>1950304405</v>
+        <v>116900000</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>-894727010</v>
+        <v>-2728131415</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>68.55124322063065</v>
+        <v>4.108917721739815</v>
       </c>
     </row>
     <row r="63">
@@ -2780,10 +2780,10 @@
         <v>1480466441</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>365280931</v>
+        <v>0</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>0</v>
@@ -2792,16 +2792,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>365280931</v>
+        <v>0</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>-1115185510</v>
+        <v>-1480466441</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>24.67336785785339</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -2817,10 +2817,10 @@
         <v>338454320</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>338454320</v>
+        <v>0</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>0</v>
@@ -2829,16 +2829,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>338454320</v>
+        <v>0</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>0</v>
+        <v>-338454320</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -2854,10 +2854,10 @@
         <v>887410440</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>1222493061</v>
+        <v>0</v>
       </c>
       <c r="F65" s="3" t="n">
         <v>0</v>
@@ -2866,16 +2866,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>1222493061</v>
+        <v>0</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>335082621</v>
+        <v>-887410440</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>137.7595987038422</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -2891,10 +2891,10 @@
         <v>1503461462</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>342919887</v>
+        <v>0</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>0</v>
@@ -2903,16 +2903,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>342919887</v>
+        <v>0</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>-1160541575</v>
+        <v>-1503461462</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>22.80869152068761</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -2928,10 +2928,10 @@
         <v>1116362329</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>1116362329</v>
+        <v>0</v>
       </c>
       <c r="F67" s="3" t="n">
         <v>0</v>
@@ -2940,16 +2940,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>1116362329</v>
+        <v>0</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>0</v>
+        <v>-1116362329</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -2965,10 +2965,10 @@
         <v>509262312</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>509262312</v>
+        <v>0</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>0</v>
@@ -2977,16 +2977,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>509262312</v>
+        <v>0</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>0</v>
+        <v>-509262312</v>
       </c>
       <c r="K68" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -3002,10 +3002,10 @@
         <v>373421530</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>373421530</v>
+        <v>0</v>
       </c>
       <c r="F69" s="3" t="n">
         <v>0</v>
@@ -3014,16 +3014,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>373421530</v>
+        <v>0</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>0</v>
+        <v>-373421530</v>
       </c>
       <c r="K69" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -3039,10 +3039,10 @@
         <v>552591787</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>552591787</v>
+        <v>0</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>0</v>
@@ -3051,16 +3051,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>552591787</v>
+        <v>0</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>0</v>
+        <v>-552591787</v>
       </c>
       <c r="K70" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -3076,10 +3076,10 @@
         <v>735655752</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>541055752</v>
+        <v>0</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>1</v>
@@ -3088,16 +3088,16 @@
         <v>194600000</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>735655752</v>
+        <v>194600000</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>0</v>
+        <v>-541055752</v>
       </c>
       <c r="K71" s="4" t="n">
-        <v>100</v>
+        <v>26.45259001522767</v>
       </c>
     </row>
     <row r="72">
@@ -3113,10 +3113,10 @@
         <v>289499767</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>289499767</v>
+        <v>0</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>0</v>
@@ -3125,16 +3125,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>289499767</v>
+        <v>0</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>0</v>
+        <v>-289499767</v>
       </c>
       <c r="K72" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -3150,10 +3150,10 @@
         <v>1774670067</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>429267455</v>
+        <v>0</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>0</v>
@@ -3162,16 +3162,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>429267455</v>
+        <v>0</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>-1345402612</v>
+        <v>-1774670067</v>
       </c>
       <c r="K73" s="4" t="n">
-        <v>24.18857809021693</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -3187,10 +3187,10 @@
         <v>1244591706</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>200070473</v>
+        <v>0</v>
       </c>
       <c r="F74" s="3" t="n">
         <v>0</v>
@@ -3199,16 +3199,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>200070473</v>
+        <v>0</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>-1044521233</v>
+        <v>-1244591706</v>
       </c>
       <c r="K74" s="4" t="n">
-        <v>16.0751893199584</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -3224,10 +3224,10 @@
         <v>329330796</v>
       </c>
       <c r="D75" s="3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>329330796</v>
+        <v>0</v>
       </c>
       <c r="F75" s="3" t="n">
         <v>0</v>
@@ -3236,16 +3236,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I75" s="3" t="n">
-        <v>329330796</v>
+        <v>0</v>
       </c>
       <c r="J75" s="3" t="n">
-        <v>0</v>
+        <v>-329330796</v>
       </c>
       <c r="K75" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -3261,10 +3261,10 @@
         <v>270659900</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>270659900</v>
+        <v>0</v>
       </c>
       <c r="F76" s="3" t="n">
         <v>0</v>
@@ -3273,16 +3273,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>270659900</v>
+        <v>0</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>0</v>
+        <v>-270659900</v>
       </c>
       <c r="K76" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -3298,10 +3298,10 @@
         <v>2453028813</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>654395500</v>
+        <v>0</v>
       </c>
       <c r="F77" s="3" t="n">
         <v>0</v>
@@ -3310,16 +3310,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>654395500</v>
+        <v>0</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>-1798633313</v>
+        <v>-2453028813</v>
       </c>
       <c r="K77" s="4" t="n">
-        <v>26.67704091089288</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -3335,10 +3335,10 @@
         <v>448879549</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>448879549</v>
+        <v>0</v>
       </c>
       <c r="F78" s="3" t="n">
         <v>0</v>
@@ -3347,16 +3347,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>448879549</v>
+        <v>0</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>0</v>
+        <v>-448879549</v>
       </c>
       <c r="K78" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -3372,10 +3372,10 @@
         <v>355094901</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>355094901</v>
+        <v>0</v>
       </c>
       <c r="F79" s="3" t="n">
         <v>0</v>
@@ -3384,16 +3384,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>355094901</v>
+        <v>0</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>0</v>
+        <v>-355094901</v>
       </c>
       <c r="K79" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -3446,10 +3446,10 @@
         <v>1301997890</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>715716850</v>
+        <v>0</v>
       </c>
       <c r="F81" s="3" t="n">
         <v>0</v>
@@ -3458,16 +3458,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>715716850</v>
+        <v>0</v>
       </c>
       <c r="J81" s="3" t="n">
-        <v>-586281040</v>
+        <v>-1301997890</v>
       </c>
       <c r="K81" s="4" t="n">
-        <v>54.97066128117919</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -3483,10 +3483,10 @@
         <v>93454644628</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>92156630628</v>
+        <v>0</v>
       </c>
       <c r="F82" s="3" t="n">
         <v>0</v>
@@ -3495,16 +3495,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="I82" s="3" t="n">
-        <v>92156630628</v>
+        <v>0</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>-1298014000</v>
+        <v>-93454644628</v>
       </c>
       <c r="K82" s="4" t="n">
-        <v>98.61107598753728</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -3520,10 +3520,10 @@
         <v>1152144239</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>1028700867</v>
+        <v>0</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>0</v>
@@ -3532,16 +3532,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="I83" s="3" t="n">
-        <v>1028700867</v>
+        <v>0</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>-123443372</v>
+        <v>-1152144239</v>
       </c>
       <c r="K83" s="4" t="n">
-        <v>89.28577101534246</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -3557,10 +3557,10 @@
         <v>19575727920</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>139</v>
+        <v>0</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>7982618589</v>
+        <v>0</v>
       </c>
       <c r="F84" s="3" t="n">
         <v>2</v>
@@ -3569,16 +3569,16 @@
         <v>350000000</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>141</v>
+        <v>2</v>
       </c>
       <c r="I84" s="3" t="n">
-        <v>8332618589</v>
+        <v>350000000</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>-11243109331</v>
+        <v>-19225727920</v>
       </c>
       <c r="K84" s="4" t="n">
-        <v>42.56607275628706</v>
+        <v>1.787928405167577</v>
       </c>
     </row>
     <row r="85">
@@ -3594,10 +3594,10 @@
         <v>17556669062</v>
       </c>
       <c r="D85" s="3" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>8306417762</v>
+        <v>0</v>
       </c>
       <c r="F85" s="3" t="n">
         <v>2</v>
@@ -3606,16 +3606,16 @@
         <v>175788800</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>170</v>
+        <v>2</v>
       </c>
       <c r="I85" s="3" t="n">
-        <v>8482206562</v>
+        <v>175788800</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>-9074462500</v>
+        <v>-17380880262</v>
       </c>
       <c r="K85" s="4" t="n">
-        <v>48.3133020964612</v>
+        <v>1.001265099770438</v>
       </c>
     </row>
     <row r="86">

</xml_diff>

<commit_message>
Auto update RUP 2026-10-20 10:39:12
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-10-20).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-10-20).xlsx
@@ -523,10 +523,10 @@
         <v>3445475044</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0</v>
+        <v>799661284</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>4</v>
@@ -535,16 +535,16 @@
         <v>946739000</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>4</v>
+        <v>77</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>946739000</v>
+        <v>1746400284</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>-2498736044</v>
+        <v>-1699074760</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>27.4777494513758</v>
+        <v>50.68677792460598</v>
       </c>
     </row>
     <row r="3">
@@ -560,10 +560,10 @@
         <v>1573461786</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>812087786</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0</v>
@@ -572,16 +572,16 @@
         <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0</v>
+        <v>812087786</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>-1573461786</v>
+        <v>-761374000</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>0</v>
+        <v>51.61153535634706</v>
       </c>
     </row>
     <row r="4">
@@ -597,10 +597,10 @@
         <v>1385846979</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>1385846979</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0</v>
@@ -609,16 +609,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0</v>
+        <v>1385846979</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>-1385846979</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -634,10 +634,10 @@
         <v>1363592000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0</v>
+        <v>1363592000</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
@@ -646,16 +646,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0</v>
+        <v>1363592000</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>-1363592000</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -708,10 +708,10 @@
         <v>3525770642</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0</v>
+        <v>2497840402</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>5</v>
@@ -720,16 +720,16 @@
         <v>1027930240</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>5</v>
+        <v>103</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>1027930240</v>
+        <v>3525770642</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>-2497840402</v>
+        <v>0</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>29.15476769121047</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -745,10 +745,10 @@
         <v>1145858598</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0</v>
+        <v>1145858598</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
@@ -757,16 +757,16 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0</v>
+        <v>1145858598</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>-1145858598</v>
+        <v>0</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -856,10 +856,10 @@
         <v>3803059695</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0</v>
+        <v>2664973989</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0</v>
@@ -868,16 +868,16 @@
         <v>0</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0</v>
+        <v>2664973989</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>-3803059695</v>
+        <v>-1138085706</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0</v>
+        <v>70.07447168141283</v>
       </c>
     </row>
     <row r="12">
@@ -893,10 +893,10 @@
         <v>985193227</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0</v>
+        <v>892817964</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0</v>
@@ -905,16 +905,16 @@
         <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0</v>
+        <v>892817964</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>-985193227</v>
+        <v>-92375263</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>0</v>
+        <v>90.62364006690436</v>
       </c>
     </row>
     <row r="13">
@@ -967,10 +967,10 @@
         <v>27966252800</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0</v>
+        <v>4961498888</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>0</v>
@@ -979,16 +979,16 @@
         <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0</v>
+        <v>4961498888</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>-27966252800</v>
+        <v>-23004753912</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>0</v>
+        <v>17.74102137845225</v>
       </c>
     </row>
     <row r="15">
@@ -1041,10 +1041,10 @@
         <v>4398271129</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0</v>
+        <v>4293942679</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>0</v>
@@ -1053,16 +1053,16 @@
         <v>0</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0</v>
+        <v>4293942679</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>-4398271129</v>
+        <v>-104328450</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>0</v>
+        <v>97.62796683196471</v>
       </c>
     </row>
     <row r="17">
@@ -1078,10 +1078,10 @@
         <v>19312615339</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0</v>
+        <v>18065133242</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0</v>
+        <v>18065133242</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>-19312615339</v>
+        <v>-1247482097</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0</v>
+        <v>93.54058435327075</v>
       </c>
     </row>
     <row r="18">
@@ -1115,10 +1115,10 @@
         <v>2386017478</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0</v>
+        <v>2326664178</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>0</v>
@@ -1127,16 +1127,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0</v>
+        <v>2326664178</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>-2386017478</v>
+        <v>-59353300</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>0</v>
+        <v>97.51245325957332</v>
       </c>
     </row>
     <row r="19">
@@ -1152,10 +1152,10 @@
         <v>26765831792</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0</v>
+        <v>440</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0</v>
+        <v>112381136563</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>1</v>
@@ -1164,16 +1164,16 @@
         <v>35000000</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1</v>
+        <v>441</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>35000000</v>
+        <v>112416136563</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>-26730831792</v>
+        <v>85650304771</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>0.1307637299374387</v>
+        <v>419.9986663466962</v>
       </c>
     </row>
     <row r="20">
@@ -1189,10 +1189,10 @@
         <v>1187854402</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0</v>
+        <v>2122940502</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>0</v>
@@ -1201,16 +1201,16 @@
         <v>0</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0</v>
+        <v>2122940502</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>-1187854402</v>
+        <v>935086100</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>0</v>
+        <v>178.7205989577164</v>
       </c>
     </row>
     <row r="21">
@@ -1263,10 +1263,10 @@
         <v>4670181047</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0</v>
+        <v>1712312836</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>0</v>
@@ -1275,16 +1275,16 @@
         <v>0</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0</v>
+        <v>1712312836</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>-4670181047</v>
+        <v>-2957868211</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>0</v>
+        <v>36.66480632693981</v>
       </c>
     </row>
     <row r="23">
@@ -1300,10 +1300,10 @@
         <v>9426756999</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0</v>
+        <v>2146723107</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0</v>
@@ -1312,16 +1312,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0</v>
+        <v>2146723107</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>-9426756999</v>
+        <v>-7280033892</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>0</v>
+        <v>22.77265773614114</v>
       </c>
     </row>
     <row r="24">
@@ -1337,10 +1337,10 @@
         <v>762843197</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0</v>
+        <v>613888229</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>0</v>
@@ -1349,16 +1349,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>0</v>
+        <v>613888229</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>-762843197</v>
+        <v>-148954968</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>0</v>
+        <v>80.47371090339553</v>
       </c>
     </row>
     <row r="25">
@@ -1374,10 +1374,10 @@
         <v>30934229421</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0</v>
+        <v>297</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0</v>
+        <v>9626894303</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>30</v>
@@ -1386,16 +1386,16 @@
         <v>52187493800</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>30</v>
+        <v>327</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>52187493800</v>
+        <v>61814388103</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>21253264379</v>
+        <v>30880158682</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>168.7046833776051</v>
+        <v>199.8252074158237</v>
       </c>
     </row>
     <row r="26">
@@ -1411,10 +1411,10 @@
         <v>10689556601</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0</v>
+        <v>10689556601</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0</v>
@@ -1423,16 +1423,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>0</v>
+        <v>10689556601</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>-10689556601</v>
+        <v>0</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
@@ -1448,10 +1448,10 @@
         <v>3526787281</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0</v>
+        <v>8063419229</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0</v>
@@ -1460,16 +1460,16 @@
         <v>0</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>0</v>
+        <v>8063419229</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>-3526787281</v>
+        <v>4536631948</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>0</v>
+        <v>228.6335575848415</v>
       </c>
     </row>
     <row r="28">
@@ -1485,10 +1485,10 @@
         <v>5579913725</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0</v>
+        <v>11165380839</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0</v>
@@ -1497,16 +1497,16 @@
         <v>0</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>0</v>
+        <v>11165380839</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-5579913725</v>
+        <v>5585467114</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>0</v>
+        <v>200.0995246391556</v>
       </c>
     </row>
     <row r="29">
@@ -1522,10 +1522,10 @@
         <v>607018311</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0</v>
+        <v>535177291</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>0</v>
+        <v>535177291</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>-607018311</v>
+        <v>-71841020</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>0</v>
+        <v>88.16493362751294</v>
       </c>
     </row>
     <row r="30">
@@ -1559,10 +1559,10 @@
         <v>6989299594</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0</v>
+        <v>11325957961</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>2</v>
@@ -1571,16 +1571,16 @@
         <v>275000000</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>2</v>
+        <v>153</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>275000000</v>
+        <v>11600957961</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>-6714299594</v>
+        <v>4611658367</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>3.934585952447583</v>
+        <v>165.9816953755839</v>
       </c>
     </row>
     <row r="31">
@@ -1596,10 +1596,10 @@
         <v>1781989871</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0</v>
+        <v>32482515490</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0</v>
@@ -1608,16 +1608,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>0</v>
+        <v>32482515490</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>-1781989871</v>
+        <v>30700525619</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>0</v>
+        <v>1822.822678098152</v>
       </c>
     </row>
     <row r="32">
@@ -1670,10 +1670,10 @@
         <v>2401856856</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0</v>
+        <v>1787561232</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0</v>
@@ -1682,16 +1682,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0</v>
+        <v>1787561232</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>-2401856856</v>
+        <v>-614295624</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>0</v>
+        <v>74.42413678960726</v>
       </c>
     </row>
     <row r="34">
@@ -1707,10 +1707,10 @@
         <v>2150571134</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0</v>
+        <v>1353030681</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>0</v>
@@ -1719,16 +1719,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0</v>
+        <v>1353030681</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>-2150571134</v>
+        <v>-797540453</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>0</v>
+        <v>62.91494662087286</v>
       </c>
     </row>
     <row r="35">
@@ -1744,10 +1744,10 @@
         <v>7783601090</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0</v>
+        <v>1564313084</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0</v>
@@ -1756,16 +1756,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>0</v>
+        <v>1564313084</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>-7783601090</v>
+        <v>-6219288006</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>0</v>
+        <v>20.09754952639794</v>
       </c>
     </row>
     <row r="36">
@@ -1781,10 +1781,10 @@
         <v>5082238023</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0</v>
+        <v>5082238023</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0</v>
@@ -1793,16 +1793,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0</v>
+        <v>5082238023</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>-5082238023</v>
+        <v>0</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
@@ -1818,10 +1818,10 @@
         <v>3494926432</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0</v>
+        <v>188</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0</v>
+        <v>4568180877</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>3</v>
@@ -1830,16 +1830,16 @@
         <v>112860000</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>3</v>
+        <v>191</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>112860000</v>
+        <v>4681040877</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>-3382066432</v>
+        <v>1186114445</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>3.229252523504907</v>
+        <v>133.9381806191908</v>
       </c>
     </row>
     <row r="38">
@@ -1855,10 +1855,10 @@
         <v>465249566</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0</v>
+        <v>465249566</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>0</v>
@@ -1867,16 +1867,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0</v>
+        <v>465249566</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>-465249566</v>
+        <v>0</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39">
@@ -1892,10 +1892,10 @@
         <v>866968514</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0</v>
+        <v>767266958</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0</v>
@@ -1904,16 +1904,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>0</v>
+        <v>767266958</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>-866968514</v>
+        <v>-99701556</v>
       </c>
       <c r="K39" s="4" t="n">
-        <v>0</v>
+        <v>88.49997959672154</v>
       </c>
     </row>
     <row r="40">
@@ -1929,10 +1929,10 @@
         <v>1439107189</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0</v>
+        <v>758839698</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>5</v>
@@ -1941,16 +1941,16 @@
         <v>168247302</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>5</v>
+        <v>106</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>168247302</v>
+        <v>927087000</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>-1270859887</v>
+        <v>-512020189</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>11.6910889811419</v>
+        <v>64.42098316833577</v>
       </c>
     </row>
     <row r="41">
@@ -1966,10 +1966,10 @@
         <v>312595476</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0</v>
+        <v>312595476</v>
       </c>
       <c r="F41" s="3" t="n">
         <v>0</v>
@@ -1978,16 +1978,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>0</v>
+        <v>312595476</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>-312595476</v>
+        <v>0</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42">
@@ -2003,10 +2003,10 @@
         <v>219851775</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0</v>
+        <v>219851775</v>
       </c>
       <c r="F42" s="3" t="n">
         <v>0</v>
@@ -2015,16 +2015,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>0</v>
+        <v>219851775</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>-219851775</v>
+        <v>0</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43">
@@ -2558,10 +2558,10 @@
         <v>2670750030</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>2639850030</v>
       </c>
       <c r="F57" s="3" t="n">
         <v>3</v>
@@ -2570,16 +2570,16 @@
         <v>30900000</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="I57" s="3" t="n">
-        <v>30900000</v>
+        <v>2670750030</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>-2639850030</v>
+        <v>0</v>
       </c>
       <c r="K57" s="4" t="n">
-        <v>1.156978363864326</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58">
@@ -2743,10 +2743,10 @@
         <v>2845031415</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0</v>
+        <v>1833404405</v>
       </c>
       <c r="F62" s="3" t="n">
         <v>1</v>
@@ -2755,16 +2755,16 @@
         <v>116900000</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>116900000</v>
+        <v>1950304405</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>-2728131415</v>
+        <v>-894727010</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>4.108917721739815</v>
+        <v>68.55124322063065</v>
       </c>
     </row>
     <row r="63">
@@ -2780,10 +2780,10 @@
         <v>1480466441</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0</v>
+        <v>365280931</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>0</v>
@@ -2792,16 +2792,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>0</v>
+        <v>365280931</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>-1480466441</v>
+        <v>-1115185510</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>0</v>
+        <v>24.67336785785339</v>
       </c>
     </row>
     <row r="64">
@@ -2817,10 +2817,10 @@
         <v>338454320</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0</v>
+        <v>338454320</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>0</v>
@@ -2829,16 +2829,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>0</v>
+        <v>338454320</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>-338454320</v>
+        <v>0</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65">
@@ -2854,10 +2854,10 @@
         <v>887410440</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0</v>
+        <v>1222493061</v>
       </c>
       <c r="F65" s="3" t="n">
         <v>0</v>
@@ -2866,16 +2866,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>0</v>
+        <v>1222493061</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>-887410440</v>
+        <v>335082621</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>0</v>
+        <v>137.7595987038422</v>
       </c>
     </row>
     <row r="66">
@@ -2891,10 +2891,10 @@
         <v>1503461462</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0</v>
+        <v>342919887</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>0</v>
@@ -2903,16 +2903,16 @@
         <v>0</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>0</v>
+        <v>342919887</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>-1503461462</v>
+        <v>-1160541575</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>0</v>
+        <v>22.80869152068761</v>
       </c>
     </row>
     <row r="67">
@@ -2928,10 +2928,10 @@
         <v>1116362329</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0</v>
+        <v>1116362329</v>
       </c>
       <c r="F67" s="3" t="n">
         <v>0</v>
@@ -2940,16 +2940,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>0</v>
+        <v>1116362329</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>-1116362329</v>
+        <v>0</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="68">
@@ -2965,10 +2965,10 @@
         <v>509262312</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0</v>
+        <v>509262312</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>0</v>
@@ -2977,16 +2977,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>0</v>
+        <v>509262312</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>-509262312</v>
+        <v>0</v>
       </c>
       <c r="K68" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="69">
@@ -3002,10 +3002,10 @@
         <v>373421530</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0</v>
+        <v>373421530</v>
       </c>
       <c r="F69" s="3" t="n">
         <v>0</v>
@@ -3014,16 +3014,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>0</v>
+        <v>373421530</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>-373421530</v>
+        <v>0</v>
       </c>
       <c r="K69" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70">
@@ -3039,10 +3039,10 @@
         <v>552591787</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0</v>
+        <v>552591787</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>0</v>
@@ -3051,16 +3051,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>0</v>
+        <v>552591787</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>-552591787</v>
+        <v>0</v>
       </c>
       <c r="K70" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="71">
@@ -3076,10 +3076,10 @@
         <v>735655752</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0</v>
+        <v>541055752</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>1</v>
@@ -3088,16 +3088,16 @@
         <v>194600000</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>194600000</v>
+        <v>735655752</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>-541055752</v>
+        <v>0</v>
       </c>
       <c r="K71" s="4" t="n">
-        <v>26.45259001522767</v>
+        <v>100</v>
       </c>
     </row>
     <row r="72">
@@ -3113,10 +3113,10 @@
         <v>289499767</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0</v>
+        <v>289499767</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>0</v>
@@ -3125,16 +3125,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>0</v>
+        <v>289499767</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>-289499767</v>
+        <v>0</v>
       </c>
       <c r="K72" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73">
@@ -3150,10 +3150,10 @@
         <v>1774670067</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0</v>
+        <v>429267455</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>0</v>
@@ -3162,16 +3162,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>0</v>
+        <v>429267455</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>-1774670067</v>
+        <v>-1345402612</v>
       </c>
       <c r="K73" s="4" t="n">
-        <v>0</v>
+        <v>24.18857809021693</v>
       </c>
     </row>
     <row r="74">
@@ -3187,10 +3187,10 @@
         <v>1244591706</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0</v>
+        <v>200070473</v>
       </c>
       <c r="F74" s="3" t="n">
         <v>0</v>
@@ -3199,16 +3199,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>0</v>
+        <v>200070473</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>-1244591706</v>
+        <v>-1044521233</v>
       </c>
       <c r="K74" s="4" t="n">
-        <v>0</v>
+        <v>16.0751893199584</v>
       </c>
     </row>
     <row r="75">
@@ -3224,10 +3224,10 @@
         <v>329330796</v>
       </c>
       <c r="D75" s="3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>0</v>
+        <v>329330796</v>
       </c>
       <c r="F75" s="3" t="n">
         <v>0</v>
@@ -3236,16 +3236,16 @@
         <v>0</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I75" s="3" t="n">
-        <v>0</v>
+        <v>329330796</v>
       </c>
       <c r="J75" s="3" t="n">
-        <v>-329330796</v>
+        <v>0</v>
       </c>
       <c r="K75" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76">
@@ -3261,10 +3261,10 @@
         <v>270659900</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0</v>
+        <v>270659900</v>
       </c>
       <c r="F76" s="3" t="n">
         <v>0</v>
@@ -3273,16 +3273,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>0</v>
+        <v>270659900</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>-270659900</v>
+        <v>0</v>
       </c>
       <c r="K76" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="77">
@@ -3298,10 +3298,10 @@
         <v>2453028813</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>0</v>
+        <v>654395500</v>
       </c>
       <c r="F77" s="3" t="n">
         <v>0</v>
@@ -3310,16 +3310,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>0</v>
+        <v>654395500</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>-2453028813</v>
+        <v>-1798633313</v>
       </c>
       <c r="K77" s="4" t="n">
-        <v>0</v>
+        <v>26.67704091089288</v>
       </c>
     </row>
     <row r="78">
@@ -3335,10 +3335,10 @@
         <v>448879549</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>0</v>
+        <v>448879549</v>
       </c>
       <c r="F78" s="3" t="n">
         <v>0</v>
@@ -3347,16 +3347,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>0</v>
+        <v>448879549</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>-448879549</v>
+        <v>0</v>
       </c>
       <c r="K78" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="79">
@@ -3372,10 +3372,10 @@
         <v>355094901</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>0</v>
+        <v>355094901</v>
       </c>
       <c r="F79" s="3" t="n">
         <v>0</v>
@@ -3384,16 +3384,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>0</v>
+        <v>355094901</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>-355094901</v>
+        <v>0</v>
       </c>
       <c r="K79" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="80">
@@ -3446,10 +3446,10 @@
         <v>1301997890</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>0</v>
+        <v>715716850</v>
       </c>
       <c r="F81" s="3" t="n">
         <v>0</v>
@@ -3458,16 +3458,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>0</v>
+        <v>715716850</v>
       </c>
       <c r="J81" s="3" t="n">
-        <v>-1301997890</v>
+        <v>-586281040</v>
       </c>
       <c r="K81" s="4" t="n">
-        <v>0</v>
+        <v>54.97066128117919</v>
       </c>
     </row>
     <row r="82">
@@ -3483,10 +3483,10 @@
         <v>93454644628</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>0</v>
+        <v>92156630628</v>
       </c>
       <c r="F82" s="3" t="n">
         <v>0</v>
@@ -3495,16 +3495,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="I82" s="3" t="n">
-        <v>0</v>
+        <v>92156630628</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>-93454644628</v>
+        <v>-1298014000</v>
       </c>
       <c r="K82" s="4" t="n">
-        <v>0</v>
+        <v>98.61107598753728</v>
       </c>
     </row>
     <row r="83">
@@ -3520,10 +3520,10 @@
         <v>1152144239</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0</v>
+        <v>1028700867</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>0</v>
@@ -3532,16 +3532,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="I83" s="3" t="n">
-        <v>0</v>
+        <v>1028700867</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>-1152144239</v>
+        <v>-123443372</v>
       </c>
       <c r="K83" s="4" t="n">
-        <v>0</v>
+        <v>89.28577101534246</v>
       </c>
     </row>
     <row r="84">
@@ -3557,10 +3557,10 @@
         <v>19575727920</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>0</v>
+        <v>7982618589</v>
       </c>
       <c r="F84" s="3" t="n">
         <v>2</v>
@@ -3569,16 +3569,16 @@
         <v>350000000</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>2</v>
+        <v>141</v>
       </c>
       <c r="I84" s="3" t="n">
-        <v>350000000</v>
+        <v>8332618589</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>-19225727920</v>
+        <v>-11243109331</v>
       </c>
       <c r="K84" s="4" t="n">
-        <v>1.787928405167577</v>
+        <v>42.56607275628706</v>
       </c>
     </row>
     <row r="85">
@@ -3594,10 +3594,10 @@
         <v>17556669062</v>
       </c>
       <c r="D85" s="3" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>0</v>
+        <v>8306417762</v>
       </c>
       <c r="F85" s="3" t="n">
         <v>2</v>
@@ -3606,16 +3606,16 @@
         <v>175788800</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="I85" s="3" t="n">
-        <v>175788800</v>
+        <v>8482206562</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>-17380880262</v>
+        <v>-9074462500</v>
       </c>
       <c r="K85" s="4" t="n">
-        <v>1.001265099770438</v>
+        <v>48.3133020964612</v>
       </c>
     </row>
     <row r="86">

</xml_diff>